<commit_message>
fix: update some datasets for the comparison
</commit_message>
<xml_diff>
--- a/examples/siwei_heme_FSEOF/heme production enhance targets.xlsx
+++ b/examples/siwei_heme_FSEOF/heme production enhance targets.xlsx
@@ -425,12 +425,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B91"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="n">
-        <v>0</v>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>k_scores</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>actions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>gene</t>
+        </is>
       </c>
     </row>
     <row r="2">
@@ -442,6 +454,16 @@
       <c r="B2" t="n">
         <v>1000</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>YLR438W</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -452,6 +474,16 @@
       <c r="B3" t="n">
         <v>1000</v>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>YBL015W</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -462,6 +494,16 @@
       <c r="B4" t="n">
         <v>1000</v>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>YHR183W</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -472,6 +514,16 @@
       <c r="B5" t="n">
         <v>1000</v>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>YNL241C</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -482,6 +534,16 @@
       <c r="B6" t="n">
         <v>1000</v>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>YLR348C</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -492,6 +554,16 @@
       <c r="B7" t="n">
         <v>1000</v>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>YKL120W</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -502,6 +574,16 @@
       <c r="B8" t="n">
         <v>1000</v>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>YER170W</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -512,26 +594,56 @@
       <c r="B9" t="n">
         <v>1000</v>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>YGR256W</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>YGR248W</t>
+          <t>YHR163W</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>1000</v>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>YHR163W</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>YHR163W</t>
+          <t>YGR248W</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>1000</v>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>YGR248W</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -542,6 +654,16 @@
       <c r="B12" t="n">
         <v>937.5625</v>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>YLR011W</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -552,6 +674,16 @@
       <c r="B13" t="n">
         <v>937.5625</v>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>YEL047C</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -562,6 +694,16 @@
       <c r="B14" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>YDR047W</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -572,6 +714,16 @@
       <c r="B15" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>YDR232W</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -582,6 +734,16 @@
       <c r="B16" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>YDR376W</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -592,6 +754,16 @@
       <c r="B17" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>YGL040C</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -602,6 +774,16 @@
       <c r="B18" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>YER014W</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -612,6 +794,16 @@
       <c r="B19" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>YPL252C</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -622,6 +814,16 @@
       <c r="B20" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>YDL205C</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -632,6 +834,16 @@
       <c r="B21" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>YPL172C</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -642,6 +854,16 @@
       <c r="B22" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>YOR278W</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -652,6 +874,16 @@
       <c r="B23" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>YMR319C</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -662,6 +894,16 @@
       <c r="B24" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>YMR058W</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
@@ -672,6 +914,16 @@
       <c r="B25" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>YOR176W</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -682,6 +934,16 @@
       <c r="B26" t="n">
         <v>700.0626297985275</v>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>YDR044W</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -692,6 +954,16 @@
       <c r="B27" t="n">
         <v>250.75</v>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>YDL171C</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -702,6 +974,16 @@
       <c r="B28" t="n">
         <v>188.3125</v>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>YKL085W</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -712,6 +994,16 @@
       <c r="B29" t="n">
         <v>42.44422062506254</v>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>YJL167W</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -722,6 +1014,16 @@
       <c r="B30" t="n">
         <v>42.44422062506254</v>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>YNR043W</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -732,6 +1034,16 @@
       <c r="B31" t="n">
         <v>42.44422062506254</v>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>YPL117C</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -742,6 +1054,16 @@
       <c r="B32" t="n">
         <v>42.44422062506254</v>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>YML126C</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -752,6 +1074,16 @@
       <c r="B33" t="n">
         <v>42.44422062506254</v>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>YML075C</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
@@ -762,6 +1094,16 @@
       <c r="B34" t="n">
         <v>42.44422062506254</v>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>YLR450W</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
@@ -772,6 +1114,16 @@
       <c r="B35" t="n">
         <v>42.44422062506254</v>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>YPL028W</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
@@ -782,6 +1134,16 @@
       <c r="B36" t="n">
         <v>42.44422062506254</v>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>YMR220W</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
@@ -792,6 +1154,16 @@
       <c r="B37" t="n">
         <v>42.44422062506227</v>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>YHR002W</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
@@ -802,6 +1174,16 @@
       <c r="B38" t="n">
         <v>8.594663605144438</v>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>YPR021C</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -812,56 +1194,116 @@
       <c r="B39" t="n">
         <v>6.611667687174141</v>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>YOL126C</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>YBR221C</t>
+          <t>YGR193C</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>4.349565727133466</v>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>YGR193C</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>YER178W</t>
+          <t>YNL071W</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>4.349565727133466</v>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>YNL071W</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>YNL071W</t>
+          <t>YBR221C</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>4.349565727133466</v>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>YBR221C</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>YGR193C</t>
+          <t>YER178W</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>4.349565727133466</v>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>YER178W</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>YCR024C-A</t>
+          <t>YPL036W</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>2.814796147504414</v>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>YPL036W</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
@@ -872,6 +1314,16 @@
       <c r="B45" t="n">
         <v>2.814796147504414</v>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>YGL008C</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
@@ -882,46 +1334,96 @@
       <c r="B46" t="n">
         <v>2.814796147504414</v>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>YEL017C-A</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>YPL036W</t>
+          <t>YCR024C-A</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>2.814796147504414</v>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>YCR024C-A</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>YBR218C</t>
+          <t>YGL062W</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>2.783360025547556</v>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>YGL062W</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>YGL062W</t>
+          <t>YBR218C</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>2.783360025547556</v>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>YBR218C</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>YHR162W</t>
+          <t>YGR243W</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>2.742569884474349</v>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>YGR243W</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
@@ -932,16 +1434,36 @@
       <c r="B51" t="n">
         <v>2.742569884474349</v>
       </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>YGL080W</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>YGR243W</t>
+          <t>YHR162W</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>2.742569884474349</v>
       </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>YHR162W</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
@@ -952,36 +1474,76 @@
       <c r="B53" t="n">
         <v>2.695197165166917</v>
       </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>YOR095C</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>YAL038W</t>
+          <t>YOR347C</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>2.485165172541028</v>
       </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>YOR347C</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>YOR347C</t>
+          <t>YAL038W</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>2.485165172541028</v>
       </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>YAL038W</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>YHR174W</t>
+          <t>YGR254W</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>2.297502885577848</v>
       </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>YGR254W</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
@@ -992,16 +1554,36 @@
       <c r="B57" t="n">
         <v>2.297502885577848</v>
       </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>YKL152C</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>YGR254W</t>
+          <t>YHR174W</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>2.297502885577848</v>
       </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>YHR174W</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
@@ -1012,6 +1594,16 @@
       <c r="B59" t="n">
         <v>1.268570038238937</v>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>YGR192C</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
@@ -1022,6 +1614,16 @@
       <c r="B60" t="n">
         <v>1.268570038238937</v>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>YJR009C</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
@@ -1032,6 +1634,16 @@
       <c r="B61" t="n">
         <v>1.268570038238937</v>
       </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>YCR012W</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
@@ -1042,6 +1654,16 @@
       <c r="B62" t="n">
         <v>1.268570038238937</v>
       </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>YJL052W</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
@@ -1052,16 +1674,36 @@
       <c r="B63" t="n">
         <v>1.207130640847328</v>
       </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>YDR050C</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>YMR205C</t>
+          <t>YGR240C</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>1.205911469528386</v>
       </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>YGR240C</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
@@ -1072,16 +1714,36 @@
       <c r="B65" t="n">
         <v>1.205911469528386</v>
       </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>YKL060C</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>YGR240C</t>
+          <t>YMR205C</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>1.205911469528386</v>
       </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>YMR205C</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
@@ -1092,6 +1754,16 @@
       <c r="B67" t="n">
         <v>1.007896475924519</v>
       </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>YPR192W</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
@@ -1102,6 +1774,16 @@
       <c r="B68" t="n">
         <v>1.007896475924519</v>
       </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>YLL052C</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
@@ -1112,6 +1794,16 @@
       <c r="B69" t="n">
         <v>0.2668744650270181</v>
       </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>YGL055W</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
@@ -1122,6 +1814,16 @@
       <c r="B70" t="n">
         <v>0.2622705785919483</v>
       </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>YKL182W</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
@@ -1132,6 +1834,16 @@
       <c r="B71" t="n">
         <v>0.2622705785919483</v>
       </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>YPL231W</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
@@ -1142,26 +1854,56 @@
       <c r="B72" t="n">
         <v>0.2618843219627576</v>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>YGL202W</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>YJR073C</t>
+          <t>YGR157W</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>0.145163841769597</v>
       </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>YGR157W</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>YGR157W</t>
+          <t>YJR073C</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>0.145163841769597</v>
       </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>YJR073C</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
@@ -1172,6 +1914,16 @@
       <c r="B75" t="n">
         <v>0.144323891078921</v>
       </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>YNL169C</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
@@ -1182,6 +1934,16 @@
       <c r="B76" t="n">
         <v>0.1439907248752916</v>
       </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>YER026C</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
@@ -1192,6 +1954,16 @@
       <c r="B77" t="n">
         <v>0.1429458713728245</v>
       </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>YBR029C</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
@@ -1202,6 +1974,16 @@
       <c r="B78" t="n">
         <v>0.1428696309914363</v>
       </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>YOR175C</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
@@ -1212,6 +1994,16 @@
       <c r="B79" t="n">
         <v>0.1428696309914363</v>
       </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>YKR067W</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
@@ -1222,6 +2014,16 @@
       <c r="B80" t="n">
         <v>0.01442493766538128</v>
       </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>YKL029C</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
@@ -1232,26 +2034,56 @@
       <c r="B81" t="n">
         <v>0</v>
       </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>YJR095W</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>YNL037C</t>
+          <t>YOR136W</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>0</v>
       </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>YOR136W</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>YOR136W</t>
+          <t>YNL037C</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>0</v>
       </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>YNL037C</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
@@ -1262,6 +2094,16 @@
       <c r="B84" t="n">
         <v>0</v>
       </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>YBR263W</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
@@ -1272,26 +2114,56 @@
       <c r="B85" t="n">
         <v>0</v>
       </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>YDL052C</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>YMR189W</t>
+          <t>YAL044C</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>0</v>
       </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>YAL044C</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>YAL044C</t>
+          <t>YDR019C</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>0</v>
       </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>YDR019C</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
@@ -1302,16 +2174,36 @@
       <c r="B88" t="n">
         <v>0</v>
       </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>YDR300C</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>YDR019C</t>
+          <t>YMR189W</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>0</v>
       </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>YMR189W</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
@@ -1322,6 +2214,16 @@
       <c r="B90" t="n">
         <v>0</v>
       </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>YMR241W</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
@@ -1331,6 +2233,16 @@
       </c>
       <c r="B91" t="n">
         <v>0</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>YOR323C</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>